<commit_message>
all the features files are moved under the folder
</commit_message>
<xml_diff>
--- a/Testcases.xlsx
+++ b/Testcases.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="TC" sheetId="1" r:id="rId1"/>
+    <sheet name="Scenario" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="56">
   <si>
     <t>TC_id</t>
   </si>
@@ -835,7 +836,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>41</v>
       </c>
@@ -989,4 +990,29 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="19.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>